<commit_message>
feat: enhance report generation, file management, and system stability
- Implement conditional input file deletion and trash recovery system
- Fix \db.queryRun\ execution flow and backend route reload issues
- Add backend cleanup logic to remove orphaned journal entries upon file deletion
- Update \.gitignore\ to prevent tracking of user-generated \.xls\/\.xlsx\ files
- Add PDF download support for output reports using \pdfmake\ with built-in fonts (A3 Landscape)
- Implement UI toggle buttons for selecting between XLS and PDF download formats
- Resolve cross-origin download corruption by utilizing fetch API and explicit ArrayBuffer-to-Blob conversion
- Apply strict zip compression (\compression: true\) to backend XLSX generation to fix MS Excel compatibility errors
</commit_message>
<xml_diff>
--- a/output-app/Neraca Lajur 2026.xlsx
+++ b/output-app/Neraca Lajur 2026.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L15"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="5.83203125" customWidth="1"/>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="G7">
-        <v>4405200</v>
+        <v>837200</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -696,7 +696,7 @@
         <v/>
       </c>
       <c r="H8">
-        <v>2672600</v>
+        <v>763600</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -731,7 +731,7 @@
         <v/>
       </c>
       <c r="G9">
-        <v>502576</v>
+        <v>251288</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -769,7 +769,7 @@
         <v/>
       </c>
       <c r="G10">
-        <v>86784920001.11</v>
+        <v>43392460000.55</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -807,7 +807,7 @@
         <v/>
       </c>
       <c r="G11">
-        <v>500000</v>
+        <v>250000</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -848,7 +848,7 @@
         <v/>
       </c>
       <c r="H12">
-        <v>500000</v>
+        <v>250000</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -886,7 +886,7 @@
         <v/>
       </c>
       <c r="H13">
-        <v>86784922577.11</v>
+        <v>43392461288.55</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -903,7 +903,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Pendapatan Harga Air</v>
+        <v>Pendapatan Denda</v>
       </c>
       <c r="B14" t="str">
         <v/>
@@ -930,7 +930,7 @@
         <v/>
       </c>
       <c r="J14">
-        <v>500000</v>
+        <v>723600</v>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -941,7 +941,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Pendapatan Denda</v>
+        <v>Pemeliharaan Kendaraan</v>
       </c>
       <c r="B15" t="str">
         <v/>
@@ -964,60 +964,22 @@
       <c r="H15" t="str">
         <v/>
       </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15">
-        <v>2532600</v>
+      <c r="I15">
+        <v>400000</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
       </c>
       <c r="K15" t="str">
         <v/>
       </c>
       <c r="L15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Pemeliharaan Kendaraan</v>
-      </c>
-      <c r="B16" t="str">
-        <v/>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
-        <v/>
-      </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-      <c r="H16" t="str">
-        <v/>
-      </c>
-      <c r="I16">
-        <v>800000</v>
-      </c>
-      <c r="J16" t="str">
-        <v/>
-      </c>
-      <c r="K16" t="str">
-        <v/>
-      </c>
-      <c r="L16" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>